<commit_message>
Update Log.xlsx with new data entries
</commit_message>
<xml_diff>
--- a/data/Log.xlsx
+++ b/data/Log.xlsx
@@ -5,20 +5,31 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Garry\tase\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Garry\market_model\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42024559-476A-438F-A699-7C649539259A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B75EB30-C20D-447E-B059-D647CB35B824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -127,15 +138,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>38613</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>104869</xdr:rowOff>
+      <xdr:rowOff>85819</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -158,8 +169,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="600075" y="190500"/>
-          <a:ext cx="3677163" cy="676369"/>
+          <a:off x="581025" y="171450"/>
+          <a:ext cx="2867025" cy="676369"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -434,13 +445,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -456,11 +470,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" t="s">
+      <c r="F1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46115</v>
       </c>
@@ -476,20 +490,24 @@
       <c r="E2">
         <v>3.47E-3</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <v>4309.68</v>
+      </c>
+      <c r="G2">
+        <f>(C2-F2)/C2*100</f>
+        <v>0.85510197039235458</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
-      <c r="I3">
-        <v>4309.68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>46145</v>
       </c>
@@ -497,31 +515,38 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="I7">
+      <c r="C7">
+        <v>4367.5965577500001</v>
+      </c>
+      <c r="F7">
         <v>4356.68</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G7">
+        <f>(C7-F7)/C7*100</f>
+        <v>0.24994427955185397</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>46176</v>
       </c>
@@ -529,28 +554,28 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add breadth signal calculation to compute_signal function and update related logic
</commit_message>
<xml_diff>
--- a/data/Log.xlsx
+++ b/data/Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Garry\market_model\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B75EB30-C20D-447E-B059-D647CB35B824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858A58B7-28F9-4A07-BD79-EBBD62AAAB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>date</t>
   </si>
@@ -78,6 +78,18 @@
   </si>
   <si>
     <t>Actual</t>
+  </si>
+  <si>
+    <t>Predicted return: 0.00176729890002082</t>
+  </si>
+  <si>
+    <t>Predicted price: 4234.4904077963665</t>
+  </si>
+  <si>
+    <t>AR(1) signal: 0.0022443452896234797</t>
+  </si>
+  <si>
+    <t>Weighted stock signal: 0.0020016489259999997</t>
   </si>
 </sst>
 </file>
@@ -576,54 +588,78 @@
       <c r="A15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>46268</v>
+      </c>
+      <c r="B16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17">
+        <v>4234.4903999999997</v>
+      </c>
+      <c r="F17">
+        <v>4227.0200000000004</v>
+      </c>
+      <c r="G17">
+        <f>(C17-F17)/C17*100</f>
+        <v>0.17641792268555492</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update Log.xlsx and index_data.csv with new data entries; enhance compute_signal function with top N stocks and signal cap
</commit_message>
<xml_diff>
--- a/data/Log.xlsx
+++ b/data/Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Garry\market_model\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858A58B7-28F9-4A07-BD79-EBBD62AAAB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4662CA3B-3B8B-4F02-B0F4-01122CB96025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>date</t>
   </si>
@@ -90,6 +90,18 @@
   </si>
   <si>
     <t>Weighted stock signal: 0.0020016489259999997</t>
+  </si>
+  <si>
+    <t>AR(1) signal: -0.0014867549685643397</t>
+  </si>
+  <si>
+    <t>Predicted return: -0.0004865583312257358</t>
+  </si>
+  <si>
+    <t>Predicted price: 4185.932308305577</t>
+  </si>
+  <si>
+    <t>Weighted stock signal: 0.0001802394270000002</t>
   </si>
 </sst>
 </file>
@@ -460,9 +472,9 @@
   <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -532,15 +544,16 @@
       <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="C7">
-        <v>4367.5965577500001</v>
+      <c r="C7" t="str">
+        <f>RIGHT(B7,FIND(":",B7)+1)</f>
+        <v>4367.596557752542</v>
       </c>
       <c r="F7">
         <v>4356.68</v>
       </c>
       <c r="G7">
         <f>(C7-F7)/C7*100</f>
-        <v>0.24994427955185397</v>
+        <v>0.24994427960986915</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -571,6 +584,17 @@
       <c r="B12" t="s">
         <v>10</v>
       </c>
+      <c r="C12" t="str">
+        <f>RIGHT(B12,FIND(":",B12)+1)</f>
+        <v>4372.519196420845</v>
+      </c>
+      <c r="F12">
+        <v>4227.0200000000004</v>
+      </c>
+      <c r="G12">
+        <f>(C12-F12)/C12*100</f>
+        <v>3.3275827934600919</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
@@ -600,15 +624,16 @@
       <c r="B17" t="s">
         <v>15</v>
       </c>
-      <c r="C17">
-        <v>4234.4903999999997</v>
+      <c r="C17" t="str">
+        <f>RIGHT(B17,FIND(":",B17)+2)</f>
+        <v>4234.4904077963665</v>
       </c>
       <c r="F17">
-        <v>4227.0200000000004</v>
+        <v>4187.97</v>
       </c>
       <c r="G17">
         <f>(C17-F17)/C17*100</f>
-        <v>0.17641792268555492</v>
+        <v>1.0986069943790295</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -627,16 +652,38 @@
       <c r="A20" s="1"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
+      <c r="A21" s="1">
+        <v>46298</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="str">
+        <f>RIGHT(B22,FIND(":",B22)+1)</f>
+        <v>4185.932308305577</v>
+      </c>
+      <c r="G22">
+        <f>(C22-F22)/C22*100</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
@@ -670,6 +717,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Log.xlsx and add Git attributes
</commit_message>
<xml_diff>
--- a/data/Log.xlsx
+++ b/data/Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Garry\market_model\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD24AC77-E47C-46F6-BA49-BB2F12BEF97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175E5E28-98D7-4730-AB5C-07D93740926E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>date</t>
   </si>
@@ -156,6 +156,36 @@
   </si>
   <si>
     <t>Weighted stock signal: -0.0012197294395</t>
+  </si>
+  <si>
+    <t>Predicted return: -0.00033740183263246805</t>
+  </si>
+  <si>
+    <t>Predicted price: 4241.048579473093</t>
+  </si>
+  <si>
+    <t>AR(1) signal: 0.0007796699359188298</t>
+  </si>
+  <si>
+    <t>Weighted stock signal: -0.001082116345</t>
+  </si>
+  <si>
+    <t>17/03/2026</t>
+  </si>
+  <si>
+    <t>18/03/26</t>
+  </si>
+  <si>
+    <t>Predicted return: 0.0002643191592149955</t>
+  </si>
+  <si>
+    <t>Predicted price: 4296.245279863936</t>
+  </si>
+  <si>
+    <t>AR(1) signal: 0.002057637055537489</t>
+  </si>
+  <si>
+    <t>Weighted stock signal: -0.0009312261050000001</t>
   </si>
 </sst>
 </file>
@@ -523,10 +553,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
@@ -872,6 +902,13 @@
         <f>RIGHT(B42,FIND(":",B42)+2)</f>
         <v xml:space="preserve"> 4174.457133623132</v>
       </c>
+      <c r="F42">
+        <v>4242.4799999999996</v>
+      </c>
+      <c r="G42">
+        <f>(C42-F42)/C42*100</f>
+        <v>-1.6295020933136377</v>
+      </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
@@ -881,6 +918,71 @@
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>41</v>
+      </c>
+      <c r="C47" t="str">
+        <f>RIGHT(B47,FIND(":",B47)+2)</f>
+        <v xml:space="preserve"> 4241.048579473093</v>
+      </c>
+      <c r="F47">
+        <v>4295.1099999999997</v>
+      </c>
+      <c r="G47">
+        <f>(C47-F47)/C47*100</f>
+        <v>-1.2747182569086724</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>45</v>
+      </c>
+      <c r="B51" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>47</v>
+      </c>
+      <c r="C52" t="str">
+        <f>RIGHT(B52,FIND(":",B52)+2)</f>
+        <v xml:space="preserve"> 4296.245279863936</v>
+      </c>
+      <c r="G52">
+        <f>(C52-F52)/C52*100</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>